<commit_message>
Updated codes in EN.variableType
</commit_message>
<xml_diff>
--- a/CEF and SCF formats/Example1_CEF_v17.xlsx
+++ b/CEF and SCF formats/Example1_CEF_v17.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icesit-my.sharepoint.com/personal/henrikkn_ices_dk/Documents/RDBES/Development/CEF SCF format/2026 02 27 CEF SCF Final uploaded to GitHub public/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk-my.sharepoint.com/personal/kibi_dtu_dk/Documents/RDBES_gits/RDBES/CEF and SCF formats/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="13_ncr:1_{3357AFD5-53AA-4CCC-B8FA-F1E38D64A2A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51691F96-1E9B-4216-969A-E6339456600E}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{3357AFD5-53AA-4CCC-B8FA-F1E38D64A2A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02822EA5-C69F-4E1B-987A-69BA0AEF2594}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{AADED950-0258-476E-8535-BAC5F529B3CA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{AADED950-0258-476E-8535-BAC5F529B3CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Catch (CN)" sheetId="1" r:id="rId1"/>
@@ -282,9 +282,6 @@
     <t>EN</t>
   </si>
   <si>
-    <t>kWd</t>
-  </si>
-  <si>
     <t>SN</t>
   </si>
   <si>
@@ -292,6 +289,9 @@
   </si>
   <si>
     <t>originType</t>
+  </si>
+  <si>
+    <t>kWd-at-sea</t>
   </si>
 </sst>
 </file>
@@ -1760,38 +1760,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F02A2425-3ED5-4099-91CA-390E20A905F1}">
   <dimension ref="A1:AA38"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.40625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.40625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.40625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="44.40625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="44.44140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="31" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.86328125" customWidth="1"/>
-    <col min="14" max="14" width="11.40625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="26.40625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="36.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="41.1328125" customWidth="1"/>
-    <col min="19" max="19" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.86328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.40625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.7265625" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.1328125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.88671875" customWidth="1"/>
+    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="36.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="41.109375" customWidth="1"/>
+    <col min="19" max="19" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.109375" style="4" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="16" style="4" customWidth="1"/>
-    <col min="25" max="25" width="11.86328125" style="4" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.88671875" style="4" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="12" style="4" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:27" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>72</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>16</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>17</v>
@@ -1874,7 +1874,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:27" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:27" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>73</v>
       </c>
@@ -1912,7 +1912,7 @@
         <v>37</v>
       </c>
       <c r="N2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O2" s="7" t="s">
         <v>38</v>
@@ -1933,7 +1933,7 @@
       <c r="X2" s="2"/>
       <c r="Z2" s="2"/>
     </row>
-    <row r="3" spans="1:27" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:27" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>73</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O3" t="s">
         <v>32</v>
@@ -1996,7 +1996,7 @@
       <c r="X3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:27" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>73</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>31</v>
       </c>
       <c r="N4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O4" t="s">
         <v>32</v>
@@ -2068,7 +2068,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>73</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O5" t="s">
         <v>32</v>
@@ -2133,7 +2133,7 @@
       <c r="Y5"/>
       <c r="Z5"/>
     </row>
-    <row r="6" spans="1:27" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>73</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>31</v>
       </c>
       <c r="N6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O6" t="s">
         <v>32</v>
@@ -2198,7 +2198,7 @@
       <c r="Y6"/>
       <c r="Z6"/>
     </row>
-    <row r="7" spans="1:27" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>73</v>
       </c>
@@ -2236,7 +2236,7 @@
         <v>31</v>
       </c>
       <c r="N7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O7" t="s">
         <v>32</v>
@@ -2263,7 +2263,7 @@
       <c r="Y7"/>
       <c r="Z7"/>
     </row>
-    <row r="8" spans="1:27" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>73</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O8" t="s">
         <v>32</v>
@@ -2328,7 +2328,7 @@
       <c r="Y8"/>
       <c r="Z8"/>
     </row>
-    <row r="9" spans="1:27" ht="18" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:27" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>73</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O9" t="s">
         <v>32</v>
@@ -2393,7 +2393,7 @@
       <c r="Y9"/>
       <c r="Z9"/>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="P10" s="3"/>
       <c r="T10" s="4"/>
       <c r="U10" s="4"/>
@@ -2401,7 +2401,7 @@
       <c r="Y10"/>
       <c r="Z10"/>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="P11" s="3"/>
       <c r="T11" s="4"/>
       <c r="U11" s="4"/>
@@ -2409,7 +2409,7 @@
       <c r="Y11"/>
       <c r="Z11"/>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="P12" s="3"/>
       <c r="T12" s="4"/>
       <c r="U12" s="4"/>
@@ -2417,7 +2417,7 @@
       <c r="Y12"/>
       <c r="Z12"/>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="P13" s="3"/>
       <c r="T13" s="4"/>
       <c r="U13" s="4"/>
@@ -2425,7 +2425,7 @@
       <c r="Y13"/>
       <c r="Z13"/>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="P14" s="3"/>
       <c r="T14" s="4"/>
       <c r="U14" s="4"/>
@@ -2433,7 +2433,7 @@
       <c r="Y14"/>
       <c r="Z14"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="P15" s="3"/>
       <c r="T15" s="4"/>
       <c r="U15" s="4"/>
@@ -2441,45 +2441,45 @@
       <c r="Y15"/>
       <c r="Z15"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="P16" s="3"/>
       <c r="X16"/>
       <c r="Y16"/>
       <c r="Z16"/>
     </row>
-    <row r="17" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="17" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P17" s="3"/>
     </row>
-    <row r="18" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="18" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P18" s="3"/>
     </row>
-    <row r="19" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="19" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P19" s="3"/>
       <c r="X19"/>
       <c r="Y19"/>
       <c r="Z19"/>
     </row>
-    <row r="20" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="20" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P20" s="3"/>
       <c r="X20"/>
       <c r="Y20"/>
       <c r="Z20"/>
     </row>
-    <row r="21" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="21" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P21" s="3"/>
       <c r="W21"/>
       <c r="X21"/>
       <c r="Y21"/>
       <c r="Z21"/>
     </row>
-    <row r="22" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="22" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P22" s="3"/>
       <c r="W22"/>
       <c r="X22"/>
       <c r="Y22"/>
       <c r="Z22"/>
     </row>
-    <row r="23" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="23" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P23" s="3"/>
       <c r="Q23" s="3"/>
       <c r="W23"/>
@@ -2487,10 +2487,10 @@
       <c r="Y23"/>
       <c r="Z23"/>
     </row>
-    <row r="24" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="24" spans="16:26" x14ac:dyDescent="0.3">
       <c r="Q24" s="3"/>
     </row>
-    <row r="25" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="25" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P25" s="3"/>
       <c r="Q25" s="3"/>
       <c r="W25"/>
@@ -2498,72 +2498,72 @@
       <c r="Y25"/>
       <c r="Z25"/>
     </row>
-    <row r="26" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="26" spans="16:26" x14ac:dyDescent="0.3">
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
     </row>
-    <row r="27" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="27" spans="16:26" x14ac:dyDescent="0.3">
       <c r="T27" s="3"/>
       <c r="U27" s="3"/>
       <c r="V27" s="5"/>
     </row>
-    <row r="28" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="28" spans="16:26" x14ac:dyDescent="0.3">
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
       <c r="V28" s="5"/>
     </row>
-    <row r="29" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="29" spans="16:26" x14ac:dyDescent="0.3">
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
       <c r="V29" s="5"/>
     </row>
-    <row r="30" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="30" spans="16:26" x14ac:dyDescent="0.3">
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
       <c r="V30" s="5"/>
     </row>
-    <row r="31" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="31" spans="16:26" x14ac:dyDescent="0.3">
       <c r="T31" s="3"/>
       <c r="U31" s="3"/>
       <c r="V31" s="5"/>
     </row>
-    <row r="32" spans="16:26" x14ac:dyDescent="0.75">
+    <row r="32" spans="16:26" x14ac:dyDescent="0.3">
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
       <c r="V32" s="5"/>
     </row>
-    <row r="33" spans="20:26" x14ac:dyDescent="0.75">
+    <row r="33" spans="20:26" x14ac:dyDescent="0.3">
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
       <c r="V33" s="5"/>
     </row>
-    <row r="34" spans="20:26" x14ac:dyDescent="0.75">
+    <row r="34" spans="20:26" x14ac:dyDescent="0.3">
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
       <c r="V34" s="5"/>
     </row>
-    <row r="35" spans="20:26" x14ac:dyDescent="0.75">
+    <row r="35" spans="20:26" x14ac:dyDescent="0.3">
       <c r="V35" s="5"/>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
       <c r="Y35" s="3"/>
       <c r="Z35" s="3"/>
     </row>
-    <row r="36" spans="20:26" x14ac:dyDescent="0.75">
+    <row r="36" spans="20:26" x14ac:dyDescent="0.3">
       <c r="V36" s="5"/>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
       <c r="Y36" s="3"/>
       <c r="Z36" s="3"/>
     </row>
-    <row r="37" spans="20:26" x14ac:dyDescent="0.75">
+    <row r="37" spans="20:26" x14ac:dyDescent="0.3">
       <c r="V37" s="5"/>
       <c r="W37" s="3"/>
       <c r="X37" s="5"/>
       <c r="Y37" s="5"/>
       <c r="Z37" s="5"/>
     </row>
-    <row r="38" spans="20:26" x14ac:dyDescent="0.75">
+    <row r="38" spans="20:26" x14ac:dyDescent="0.3">
       <c r="V38" s="5"/>
       <c r="X38" s="5"/>
       <c r="Y38" s="5"/>
@@ -2582,34 +2582,34 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF2838F0-2BB3-41FA-8710-A7D3F89C1665}">
   <dimension ref="A1:W60"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.86328125" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.54296875" customWidth="1"/>
-    <col min="6" max="6" width="14.7265625" customWidth="1"/>
-    <col min="7" max="7" width="19.86328125" customWidth="1"/>
-    <col min="8" max="8" width="40.26953125" customWidth="1"/>
-    <col min="9" max="9" width="16.40625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.86328125" customWidth="1"/>
-    <col min="14" max="14" width="15.40625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.86328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.86328125" customWidth="1"/>
-    <col min="17" max="17" width="15.86328125" customWidth="1"/>
-    <col min="18" max="18" width="11.40625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17.40625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.40625" customWidth="1"/>
-    <col min="21" max="21" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" customWidth="1"/>
+    <col min="6" max="6" width="14.77734375" customWidth="1"/>
+    <col min="7" max="7" width="19.88671875" customWidth="1"/>
+    <col min="8" max="8" width="40.21875" customWidth="1"/>
+    <col min="9" max="9" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.88671875" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.88671875" customWidth="1"/>
+    <col min="17" max="17" width="15.88671875" customWidth="1"/>
+    <col min="18" max="18" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.44140625" customWidth="1"/>
+    <col min="21" max="21" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:23" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>72</v>
       </c>
@@ -2680,7 +2680,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>75</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>75</v>
       </c>
@@ -2810,7 +2810,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -2875,7 +2875,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>75</v>
       </c>
@@ -2940,7 +2940,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -3005,7 +3005,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -3070,7 +3070,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>75</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>75</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>75</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>75</v>
       </c>
@@ -3330,7 +3330,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>75</v>
       </c>
@@ -3395,7 +3395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>75</v>
       </c>
@@ -3460,7 +3460,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>75</v>
       </c>
@@ -3525,7 +3525,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>75</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>75</v>
       </c>
@@ -3655,7 +3655,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>75</v>
       </c>
@@ -3720,7 +3720,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>75</v>
       </c>
@@ -3785,7 +3785,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>75</v>
       </c>
@@ -3850,7 +3850,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>75</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>75</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>75</v>
       </c>
@@ -4045,7 +4045,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>75</v>
       </c>
@@ -4110,7 +4110,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -4175,7 +4175,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>75</v>
       </c>
@@ -4240,7 +4240,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>75</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>75</v>
       </c>
@@ -4435,7 +4435,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>75</v>
       </c>
@@ -4500,7 +4500,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
@@ -4509,7 +4509,7 @@
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.75">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
@@ -4518,7 +4518,7 @@
       <c r="V32" s="3"/>
       <c r="W32" s="3"/>
     </row>
-    <row r="33" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="33" spans="7:23" x14ac:dyDescent="0.3">
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
@@ -4527,7 +4527,7 @@
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
     </row>
-    <row r="34" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="34" spans="7:23" x14ac:dyDescent="0.3">
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
@@ -4536,7 +4536,7 @@
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
     </row>
-    <row r="35" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="35" spans="7:23" x14ac:dyDescent="0.3">
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
@@ -4545,7 +4545,7 @@
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
     </row>
-    <row r="36" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="36" spans="7:23" x14ac:dyDescent="0.3">
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
@@ -4554,7 +4554,7 @@
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
     </row>
-    <row r="37" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="37" spans="7:23" x14ac:dyDescent="0.3">
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
       <c r="K37" s="3"/>
@@ -4563,7 +4563,7 @@
       <c r="V37" s="3"/>
       <c r="W37" s="3"/>
     </row>
-    <row r="38" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="38" spans="7:23" x14ac:dyDescent="0.3">
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
@@ -4572,7 +4572,7 @@
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
     </row>
-    <row r="39" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="39" spans="7:23" x14ac:dyDescent="0.3">
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
@@ -4581,7 +4581,7 @@
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
     </row>
-    <row r="40" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="40" spans="7:23" x14ac:dyDescent="0.3">
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
@@ -4590,140 +4590,140 @@
       <c r="V40" s="3"/>
       <c r="W40" s="3"/>
     </row>
-    <row r="41" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="41" spans="7:23" x14ac:dyDescent="0.3">
       <c r="H41" s="6"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
       <c r="V41" s="3"/>
       <c r="W41" s="3"/>
     </row>
-    <row r="42" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="42" spans="7:23" x14ac:dyDescent="0.3">
       <c r="G42" s="6"/>
       <c r="S42" s="3"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
     </row>
-    <row r="43" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="43" spans="7:23" x14ac:dyDescent="0.3">
       <c r="G43" s="6"/>
       <c r="S43" s="3"/>
       <c r="T43" s="3"/>
       <c r="U43" s="3"/>
       <c r="V43" s="3"/>
     </row>
-    <row r="44" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="44" spans="7:23" x14ac:dyDescent="0.3">
       <c r="G44" s="6"/>
       <c r="S44" s="3"/>
       <c r="T44" s="3"/>
       <c r="U44" s="3"/>
       <c r="V44" s="3"/>
     </row>
-    <row r="45" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="45" spans="7:23" x14ac:dyDescent="0.3">
       <c r="G45" s="6"/>
       <c r="S45" s="3"/>
       <c r="T45" s="3"/>
       <c r="U45" s="3"/>
       <c r="V45" s="3"/>
     </row>
-    <row r="46" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="46" spans="7:23" x14ac:dyDescent="0.3">
       <c r="G46" s="6"/>
       <c r="S46" s="3"/>
       <c r="T46" s="3"/>
       <c r="U46" s="3"/>
       <c r="V46" s="3"/>
     </row>
-    <row r="47" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="47" spans="7:23" x14ac:dyDescent="0.3">
       <c r="G47" s="6"/>
       <c r="S47" s="3"/>
       <c r="T47" s="3"/>
       <c r="U47" s="3"/>
       <c r="V47" s="3"/>
     </row>
-    <row r="48" spans="7:23" x14ac:dyDescent="0.75">
+    <row r="48" spans="7:23" x14ac:dyDescent="0.3">
       <c r="G48" s="6"/>
       <c r="S48" s="3"/>
       <c r="T48" s="3"/>
       <c r="U48" s="3"/>
       <c r="V48" s="3"/>
     </row>
-    <row r="49" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="49" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G49" s="6"/>
       <c r="S49" s="3"/>
       <c r="T49" s="3"/>
       <c r="U49" s="3"/>
       <c r="V49" s="3"/>
     </row>
-    <row r="50" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="50" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G50" s="6"/>
       <c r="S50" s="3"/>
       <c r="T50" s="3"/>
       <c r="U50" s="3"/>
       <c r="V50" s="3"/>
     </row>
-    <row r="51" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="51" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G51" s="6"/>
       <c r="S51" s="3"/>
       <c r="T51" s="3"/>
       <c r="U51" s="3"/>
       <c r="V51" s="3"/>
     </row>
-    <row r="52" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="52" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G52" s="6"/>
       <c r="S52" s="3"/>
       <c r="T52" s="3"/>
       <c r="U52" s="3"/>
       <c r="V52" s="3"/>
     </row>
-    <row r="53" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="53" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G53" s="6"/>
       <c r="S53" s="3"/>
       <c r="T53" s="3"/>
       <c r="U53" s="3"/>
       <c r="V53" s="3"/>
     </row>
-    <row r="54" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="54" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G54" s="6"/>
       <c r="S54" s="3"/>
       <c r="T54" s="3"/>
       <c r="U54" s="3"/>
       <c r="V54" s="3"/>
     </row>
-    <row r="55" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="55" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G55" s="6"/>
       <c r="S55" s="3"/>
       <c r="T55" s="3"/>
       <c r="U55" s="3"/>
       <c r="V55" s="3"/>
     </row>
-    <row r="56" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="56" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G56" s="6"/>
       <c r="S56" s="3"/>
       <c r="T56" s="3"/>
       <c r="U56" s="3"/>
       <c r="V56" s="3"/>
     </row>
-    <row r="57" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="57" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G57" s="6"/>
       <c r="S57" s="3"/>
       <c r="T57" s="3"/>
       <c r="U57" s="3"/>
       <c r="V57" s="3"/>
     </row>
-    <row r="58" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="58" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G58" s="6"/>
       <c r="S58" s="3"/>
       <c r="T58" s="3"/>
       <c r="U58" s="3"/>
       <c r="V58" s="3"/>
     </row>
-    <row r="59" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="59" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G59" s="6"/>
       <c r="S59" s="3"/>
       <c r="T59" s="3"/>
       <c r="U59" s="3"/>
       <c r="V59" s="3"/>
     </row>
-    <row r="60" spans="7:22" x14ac:dyDescent="0.75">
+    <row r="60" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G60" s="6"/>
       <c r="S60" s="3"/>
       <c r="T60" s="3"/>
@@ -4742,26 +4742,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{103B734F-23CA-4FDD-9D43-E5DB8E886C55}">
   <dimension ref="A1:O17"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.26953125" customWidth="1"/>
-    <col min="2" max="2" width="21.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.40625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.40625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.40625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.86328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.21875" customWidth="1"/>
+    <col min="2" max="2" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.5546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28.54296875" customWidth="1"/>
-    <col min="13" max="13" width="15.1328125" customWidth="1"/>
-    <col min="14" max="14" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.5546875" customWidth="1"/>
+    <col min="13" max="13" width="15.109375" customWidth="1"/>
+    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:15" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>72</v>
       </c>
@@ -4799,7 +4799,7 @@
         <v>13</v>
       </c>
       <c r="M1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N1" t="s">
         <v>17</v>
@@ -4808,7 +4808,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -4837,7 +4837,7 @@
         <v>37</v>
       </c>
       <c r="K2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L2" s="7" t="s">
         <v>38</v>
@@ -4846,13 +4846,13 @@
         <v>74</v>
       </c>
       <c r="N2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O2">
         <v>369841</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -4881,7 +4881,7 @@
         <v>31</v>
       </c>
       <c r="K3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>32</v>
@@ -4890,13 +4890,13 @@
         <v>74</v>
       </c>
       <c r="N3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O3">
         <v>235931</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -4925,7 +4925,7 @@
         <v>31</v>
       </c>
       <c r="K4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>32</v>
@@ -4934,13 +4934,13 @@
         <v>74</v>
       </c>
       <c r="N4" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O4">
         <v>478521</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -4969,7 +4969,7 @@
         <v>31</v>
       </c>
       <c r="K5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>32</v>
@@ -4978,13 +4978,13 @@
         <v>74</v>
       </c>
       <c r="N5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O5">
         <v>213694</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -5013,7 +5013,7 @@
         <v>31</v>
       </c>
       <c r="K6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>32</v>
@@ -5022,13 +5022,13 @@
         <v>74</v>
       </c>
       <c r="N6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O6">
         <v>258963</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>78</v>
       </c>
@@ -5057,7 +5057,7 @@
         <v>31</v>
       </c>
       <c r="K7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>32</v>
@@ -5066,13 +5066,13 @@
         <v>74</v>
       </c>
       <c r="N7" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O7">
         <v>256987</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>78</v>
       </c>
@@ -5101,7 +5101,7 @@
         <v>31</v>
       </c>
       <c r="K8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>32</v>
@@ -5110,13 +5110,13 @@
         <v>74</v>
       </c>
       <c r="N8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O8">
         <v>25639</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>31</v>
       </c>
       <c r="K9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>32</v>
@@ -5154,13 +5154,13 @@
         <v>74</v>
       </c>
       <c r="N9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O9">
         <v>24785</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -5189,7 +5189,7 @@
         <v>31</v>
       </c>
       <c r="K10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>32</v>
@@ -5198,13 +5198,13 @@
         <v>74</v>
       </c>
       <c r="N10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O10">
         <v>123654</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>78</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>31</v>
       </c>
       <c r="K11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>32</v>
@@ -5242,13 +5242,13 @@
         <v>74</v>
       </c>
       <c r="N11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O11">
         <v>14789</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>78</v>
       </c>
@@ -5277,7 +5277,7 @@
         <v>31</v>
       </c>
       <c r="K12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L12" s="7" t="s">
         <v>32</v>
@@ -5286,13 +5286,13 @@
         <v>74</v>
       </c>
       <c r="N12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O12">
         <v>10236</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>78</v>
       </c>
@@ -5321,7 +5321,7 @@
         <v>31</v>
       </c>
       <c r="K13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L13" s="7" t="s">
         <v>32</v>
@@ -5330,13 +5330,13 @@
         <v>74</v>
       </c>
       <c r="N13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O13">
         <v>25804</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -5365,7 +5365,7 @@
         <v>31</v>
       </c>
       <c r="K14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L14" s="7" t="s">
         <v>32</v>
@@ -5374,13 +5374,13 @@
         <v>74</v>
       </c>
       <c r="N14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O14">
         <v>12369</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>78</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>31</v>
       </c>
       <c r="K15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L15" s="7" t="s">
         <v>32</v>
@@ -5418,13 +5418,13 @@
         <v>74</v>
       </c>
       <c r="N15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O15">
         <v>25896</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>78</v>
       </c>
@@ -5453,7 +5453,7 @@
         <v>31</v>
       </c>
       <c r="K16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L16" s="7" t="s">
         <v>32</v>
@@ -5462,13 +5462,13 @@
         <v>74</v>
       </c>
       <c r="N16" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O16">
         <v>1245</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>78</v>
       </c>
@@ -5497,7 +5497,7 @@
         <v>31</v>
       </c>
       <c r="K17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L17" s="7" t="s">
         <v>32</v>
@@ -5506,7 +5506,7 @@
         <v>74</v>
       </c>
       <c r="N17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O17">
         <v>236987</v>
@@ -5520,32 +5520,32 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D520F06D-28E3-4BF9-BEFE-26976F39EACC}">
   <dimension ref="A1:U4"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.86328125" customWidth="1"/>
-    <col min="2" max="2" width="22.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.40625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.40625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.40625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.86328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="25.453125" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.44140625" customWidth="1"/>
     <col min="13" max="13" width="24" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="40" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.40625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27.1328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.86328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.40625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.1328125" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7.109375" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:21" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>72</v>
       </c>
@@ -5598,7 +5598,7 @@
         <v>13</v>
       </c>
       <c r="R1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S1" t="s">
         <v>17</v>
@@ -5610,9 +5610,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
         <v>24</v>
@@ -5654,7 +5654,7 @@
         <v>37</v>
       </c>
       <c r="P2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q2" s="7" t="s">
         <v>38</v>
@@ -5672,9 +5672,9 @@
         <v>250</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B3" t="s">
         <v>24</v>
@@ -5716,7 +5716,7 @@
         <v>37</v>
       </c>
       <c r="P3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q3" s="7" t="s">
         <v>38</v>
@@ -5734,9 +5734,9 @@
         <v>6350</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
@@ -5778,7 +5778,7 @@
         <v>31</v>
       </c>
       <c r="P4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q4" s="7" t="s">
         <v>32</v>
@@ -5806,6 +5806,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CF5149A2F9434B4282E37FA76C9DDAE3" ma:contentTypeVersion="0" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="926e61e4a601c985d0b7a12fe0d96524">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="500c6692915ba10984c0aabd49f31b22">
     <xsd:element name="properties">
@@ -5919,22 +5934,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95273AB9-3FE7-443B-981C-3251612C63FA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8797D6E-9AB0-436C-BF76-0F53999D6373}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BE5FEE5A-38D1-40BC-B5C2-5C0144C7FE5C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5948,27 +5971,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8797D6E-9AB0-436C-BF76-0F53999D6373}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95273AB9-3FE7-443B-981C-3251612C63FA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>